<commit_message>
Fast rebuild valuation and reports
</commit_message>
<xml_diff>
--- a/Vietnam_Banking_Equity_Valuation_MA_Master.xlsx
+++ b/Vietnam_Banking_Equity_Valuation_MA_Master.xlsx
@@ -2,20 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R46dd025ed36745c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BANK_UNIVERSE" sheetId="2" r:id="R4526b171880b4904"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VALUATION_ASSUMPTIONS" sheetId="3" r:id="R8eee7fc6c56741b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VALUATION_TEMPLATE" sheetId="4" r:id="R6f662f0fc2444a00"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M&amp;A_ASSUMPTIONS" sheetId="5" r:id="R6e6e64a939ab4fac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DEAL_SIMULATOR" sheetId="6" r:id="R4f6d64c91a484480"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DEAL_PRECEDENTS" sheetId="7" r:id="Rfd8a61c94f2f4bb5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RESTRUCTURING" sheetId="8" r:id="R04c934cd82fe4993"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GOVERNANCE" sheetId="9" r:id="R98f229d573bd430d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SOURCES" sheetId="10" r:id="R8b2fd757febf4d5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BANK_ASSUMPTIONS" sheetId="11" r:id="Rfe1752ffefcc4a2c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TRONG_SO_CHAM_DIEM" sheetId="12" r:id="R50f4378b7a3843d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAU_HINH_BAO_CAO" sheetId="13" r:id="R16800dec49ec4e25"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KIEM_SOAT_PHAT_HANH" sheetId="14" r:id="R459bbe83794f4634"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rdc1795c1ec964415"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BANK_UNIVERSE" sheetId="2" r:id="Rfdc06894de3d4f39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VALUATION_ASSUMPTIONS" sheetId="3" r:id="R11669961a63e42ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VALUATION_TEMPLATE" sheetId="4" r:id="R4214b0dd4c114004"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M&amp;A_ASSUMPTIONS" sheetId="5" r:id="R3d54348056654052"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DEAL_SIMULATOR" sheetId="6" r:id="Re52f2f0631ea4be1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DEAL_PRECEDENTS" sheetId="7" r:id="Rcb59f36acfbe4468"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RESTRUCTURING" sheetId="8" r:id="R93b99484395c4505"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GOVERNANCE" sheetId="9" r:id="Rd8365276d1144aa4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SOURCES" sheetId="10" r:id="R020fe229875f44be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BANK_ASSUMPTIONS" sheetId="11" r:id="Rc81b8d0bfb864568"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TRONG_SO_CHAM_DIEM" sheetId="12" r:id="Rc5059a8b299f4efa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAU_HINH_BAO_CAO" sheetId="13" r:id="Rda6c526371eb45fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KIEM_SOAT_PHAT_HANH" sheetId="14" r:id="R5b3c2fce8d8b4831"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BENCHMARK_20_NH" sheetId="15" r:id="Rd67feaaba7524511"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="STB_STRATEGIC_CASE" sheetId="16" r:id="R6529ab52497e4f96"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -26,13 +28,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="6">
+  <x:numFmts count="8">
     <x:numFmt numFmtId="200" formatCode="0.0%"/>
     <x:numFmt numFmtId="201" formatCode="#,##0;[Red](#,##0);-"/>
     <x:numFmt numFmtId="202" formatCode="0.0%;[Red](0.0%);-"/>
     <x:numFmt numFmtId="203" formatCode="#,##0.0;[Red](#,##0.0);-"/>
     <x:numFmt numFmtId="204" formatCode="0.00x"/>
     <x:numFmt numFmtId="205" formatCode="0%"/>
+    <x:numFmt numFmtId="206" formatCode="#,##0.0"/>
+    <x:numFmt numFmtId="207" formatCode="#,##0"/>
   </x:numFmts>
   <x:fonts count="5">
     <x:font>
@@ -62,7 +66,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="17">
+  <x:fills count="20">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -144,6 +148,21 @@
         <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F2747"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0B6E69"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -152,7 +171,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="69">
+  <x:cellXfs count="83">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -252,6 +271,24 @@
     <x:xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="205" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="3" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="207" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -397,7 +434,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R568870c465bd433c"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd862d933a8414c2d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -745,6 +782,14 @@
         <x:v>Tự kiểm tra độ phủ dữ liệu trước khi phát hành; phân loại CHÍNH THỨC / BẢN NHÁP / CHƯA ĐỦ DỮ LIỆU; đóng dấu draft trên PDF; tự phát hiện các điểm cần normalization như ROE bất thường, NPL/CAR và P/B vượt vùng hợp lý.</x:v>
       </x:c>
     </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="44" t="str">
+        <x:v>V6.2 - Việt hóa &amp; tách biểu đồ</x:v>
+      </x:c>
+      <x:c r="B19" s="43" t="str">
+        <x:v>Giao diện và báo cáo dùng nhãn tiếng Việt; mỗi chỉ tiêu lịch sử được tách thành biểu đồ riêng với đường bình quân 20 ngân hàng; trục Y có khoảng đệm tự động để tránh đường dữ liệu sát trục hoành.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
@@ -1986,6 +2031,707 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="42" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="50" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="40" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="42" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="42" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="75" t="str">
+        <x:v>BENCHMARK BÌNH QUÂN 20 NGÂN HÀNG</x:v>
+      </x:c>
+      <x:c r="B1" s="75"/>
+      <x:c r="C1" s="75"/>
+      <x:c r="D1" s="75"/>
+      <x:c r="E1" s="75"/>
+      <x:c r="F1" s="75"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="74" t="str">
+        <x:v>Hạng mục</x:v>
+      </x:c>
+      <x:c r="B3" s="74" t="str">
+        <x:v>Thiết kế</x:v>
+      </x:c>
+      <x:c r="C3" s="74" t="str">
+        <x:v>Phạm vi</x:v>
+      </x:c>
+      <x:c r="D3" s="74" t="str">
+        <x:v>Xử lý dữ liệu thiếu</x:v>
+      </x:c>
+      <x:c r="E3" s="74" t="str">
+        <x:v>Hiển thị chart</x:v>
+      </x:c>
+      <x:c r="F3" s="74" t="str">
+        <x:v>Ghi chú</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>Universe</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>20 ngân hàng trong BANK_UNIVERSE</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>VCB, BID, CTG, TCB, MBB, ACB, HDB, VPB, STB, VIB, SHB, TPB, LPB, OCB, MSB, SSB, EIB, NAB, KLB, BAB</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>Không biến N/A thành 0</x:v>
+      </x:c>
+      <x:c r="E4" t="str">
+        <x:v>Đường nét đứt 'Bình quân 20 NH'</x:v>
+      </x:c>
+      <x:c r="F4" t="str">
+        <x:v>Bình quân số học các ngân hàng có dữ liệu tại từng kỳ</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>ROE/ROA/NIM</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>Bình quân theo kỳ</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>20 NH</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>Loại N/A/0 không hợp lệ</x:v>
+      </x:c>
+      <x:c r="E5" t="str">
+        <x:v>Target solid + peer dashed</x:v>
+      </x:c>
+      <x:c r="F5" t="str">
+        <x:v>%</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>NPL/CAR/CASA/CIR/LDR</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>Bình quân theo kỳ</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>20 NH</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>Loại N/A; CAR&lt;=0 loại khỏi benchmark</x:v>
+      </x:c>
+      <x:c r="E6" t="str">
+        <x:v>Target solid + peer dashed</x:v>
+      </x:c>
+      <x:c r="F6" t="str">
+        <x:v>%</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>Tài sản/Dư nợ/Tiền gửi</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>Bình quân quy mô theo kỳ</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>20 NH</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>Loại N/A</x:v>
+      </x:c>
+      <x:c r="E7" t="str">
+        <x:v>Target solid + peer dashed</x:v>
+      </x:c>
+      <x:c r="F7" t="str">
+        <x:v>VND</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>Giá cổ phiếu</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>Chỉ số hóa đầu kỳ = 100</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>20 NH</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>Loại N/A</x:v>
+      </x:c>
+      <x:c r="E8" t="str">
+        <x:v>Target index + equal-weight average index</x:v>
+      </x:c>
+      <x:c r="F8" t="str">
+        <x:v>Không so giá tuyệt đối giữa cổ phiếu</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>ROE-P/B scatter</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>Bình quân chéo hiện tại</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>20 NH</x:v>
+      </x:c>
+      <x:c r="D9" t="str">
+        <x:v>Loại N/A</x:v>
+      </x:c>
+      <x:c r="E9" t="str">
+        <x:v>Crosshair ROE/PB bình quân</x:v>
+      </x:c>
+      <x:c r="F9" t="str"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>Thẻ điểm 6 trụ cột</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>Bình quân điểm từng trụ cột</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>20 NH</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>Loại N/A</x:v>
+      </x:c>
+      <x:c r="E10" t="str">
+        <x:v>Marker/line peer average</x:v>
+      </x:c>
+      <x:c r="F10" t="str">
+        <x:v>Điểm /100</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>Football Field</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>P/B bình quân 20 NH x BVPS ngân hàng mục tiêu</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>20 NH</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>Loại N/A</x:v>
+      </x:c>
+      <x:c r="E11" t="str">
+        <x:v>Đường benchmark peer-implied value</x:v>
+      </x:c>
+      <x:c r="F11" t="str">
+        <x:v>Không thay thế fair value nội tại</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:F1"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="56" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="80" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="24" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="75" t="str">
+        <x:v>STB - KIỂM TRA TÍNH HỢP LÝ GIÁ THÂU TÓM 80.000-100.000 ĐỒNG/CP</x:v>
+      </x:c>
+      <x:c r="B1" s="75"/>
+      <x:c r="C1" s="75"/>
+      <x:c r="D1" s="75"/>
+      <x:c r="E1" s="75"/>
+      <x:c r="F1" s="75"/>
+      <x:c r="G1" s="75"/>
+      <x:c r="H1" s="75"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="73" t="str">
+        <x:v>Đầu vào</x:v>
+      </x:c>
+      <x:c r="B3" s="73" t="str">
+        <x:v>Giá trị</x:v>
+      </x:c>
+      <x:c r="C3" s="73" t="str">
+        <x:v>Đơn vị</x:v>
+      </x:c>
+      <x:c r="D3" s="73" t="str">
+        <x:v>Lineage</x:v>
+      </x:c>
+      <x:c r="F3" s="73" t="str">
+        <x:v>Kiểm tra</x:v>
+      </x:c>
+      <x:c r="G3" s="73" t="str">
+        <x:v>80.000</x:v>
+      </x:c>
+      <x:c r="H3" s="73" t="str">
+        <x:v>100.000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>Giá thị trường STB</x:v>
+      </x:c>
+      <x:c r="B4" s="76" t="n">
+        <x:v>74.7</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>nghìn đồng/cp</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>ACTUAL snapshot</x:v>
+      </x:c>
+      <x:c r="F4" t="str">
+        <x:v>Premium so với thị giá</x:v>
+      </x:c>
+      <x:c r="G4" s="78" t="n">
+        <x:f>$B$5/$B$4-1</x:f>
+        <x:v>0.07095046854082998</x:v>
+      </x:c>
+      <x:c r="H4" s="78" t="n">
+        <x:f>$B$6/$B$4-1</x:f>
+        <x:v>0.3386880856760375</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>Giá chiến lược thấp</x:v>
+      </x:c>
+      <x:c r="B5" s="76" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>nghìn đồng/cp</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>USER_MARKET_INTELLIGENCE</x:v>
+      </x:c>
+      <x:c r="F5" t="str">
+        <x:v>P/B hiện tại</x:v>
+      </x:c>
+      <x:c r="G5" s="30" t="n">
+        <x:f>$B$5/$B$9</x:f>
+        <x:v>2.394842395571625</x:v>
+      </x:c>
+      <x:c r="H5" s="30" t="n">
+        <x:f>$B$6/$B$9</x:f>
+        <x:v>2.9935529944645314</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>Giá chiến lược cao</x:v>
+      </x:c>
+      <x:c r="B6" s="76" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>nghìn đồng/cp</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>USER_MARKET_INTELLIGENCE</x:v>
+      </x:c>
+      <x:c r="F6" t="str">
+        <x:v>P/B hậu xử lý</x:v>
+      </x:c>
+      <x:c r="G6" s="30" t="n">
+        <x:f>$B$5/($B$9+$B$10)</x:f>
+        <x:v>1.8431004949853727</x:v>
+      </x:c>
+      <x:c r="H6" s="30" t="n">
+        <x:f>$B$6/($B$9+$B$10)</x:f>
+        <x:v>2.3038756187317158</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>Tỷ lệ lô tham chiếu</x:v>
+      </x:c>
+      <x:c r="B7" s="77" t="n">
+        <x:v>0.325</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>%</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>PUBLIC/SCENARIO</x:v>
+      </x:c>
+      <x:c r="F7" t="str">
+        <x:v>Giá trị lô 32,5% (tỷ đồng)</x:v>
+      </x:c>
+      <x:c r="G7" s="22" t="n">
+        <x:f>$B$5*$B$7*$B$8*1000</x:f>
+        <x:v>48884.375384</x:v>
+      </x:c>
+      <x:c r="H7" s="22" t="n">
+        <x:f>$B$6*$B$7*$B$8*1000</x:f>
+        <x:v>61105.46923</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>Số cổ phiếu lưu hành</x:v>
+      </x:c>
+      <x:c r="B8" s="76" t="n">
+        <x:v>1.880168284</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>tỷ cp</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>CALCULATED/ACTUAL</x:v>
+      </x:c>
+      <x:c r="F8" t="str">
+        <x:v>Bao phủ 63.250 tỷ gốc+lãi</x:v>
+      </x:c>
+      <x:c r="G8" s="78" t="n">
+        <x:f>G7/$B$11</x:f>
+        <x:v>0.7728755001422924</x:v>
+      </x:c>
+      <x:c r="H8" s="78" t="n">
+        <x:f>H7/$B$11</x:f>
+        <x:v>0.9660943751778657</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>BVPS hiện tại</x:v>
+      </x:c>
+      <x:c r="B9" s="76" t="n">
+        <x:v>33.405121</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>nghìn đồng/cp</x:v>
+      </x:c>
+      <x:c r="D9" t="str">
+        <x:v>CALCULATED</x:v>
+      </x:c>
+      <x:c r="F9" t="str">
+        <x:v>Premium/(discount) high-case 81k</x:v>
+      </x:c>
+      <x:c r="G9" s="78" t="n">
+        <x:f>$B$5/$B$12-1</x:f>
+        <x:v>-0.012345679012345734</x:v>
+      </x:c>
+      <x:c r="H9" s="78" t="n">
+        <x:f>$B$6/$B$12-1</x:f>
+        <x:v>0.23456790123456783</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>Uplift BVPS hậu xử lý</x:v>
+      </x:c>
+      <x:c r="B10" s="76" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>nghìn đồng/cp</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>PUBLIC_RESEARCH_SCENARIO</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>Gốc + lãi liên quan tài sản bảo đảm</x:v>
+      </x:c>
+      <x:c r="B11" s="76" t="n">
+        <x:v>63250</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>tỷ đồng</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>PUBLIC_RESEARCH_ESTIMATE</x:v>
+      </x:c>
+      <x:c r="F11" s="73" t="str">
+        <x:v>Chỉ tiêu bổ sung</x:v>
+      </x:c>
+      <x:c r="G11" s="73" t="str">
+        <x:v>Giá trị</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>High-case standalone công khai</x:v>
+      </x:c>
+      <x:c r="B12" s="76" t="n">
+        <x:v>81</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>nghìn đồng/cp</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>PUBLIC_RESEARCH</x:v>
+      </x:c>
+      <x:c r="F12" t="str">
+        <x:v>Giá clearing cho thu hồi 100%</x:v>
+      </x:c>
+      <x:c r="G12" s="79" t="n">
+        <x:f>$B$11/($B$7*$B$8)</x:f>
+        <x:v>103509.55617725154</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="F13" t="str">
+        <x:v>Giá trị lô tại 80k</x:v>
+      </x:c>
+      <x:c r="G13" s="80" t="n">
+        <x:f>G7</x:f>
+        <x:v>48884.375384</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="F14" t="str">
+        <x:v>Giá trị lô tại 100k</x:v>
+      </x:c>
+      <x:c r="G14" s="80" t="n">
+        <x:f>H7</x:f>
+        <x:v>61105.46923</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="81" t="str">
+        <x:v>NGUỒN THAM KHẢO &amp; KẾT LUẬN</x:v>
+      </x:c>
+      <x:c r="B16" s="81"/>
+      <x:c r="C16" s="81"/>
+      <x:c r="D16" s="81"/>
+      <x:c r="E16" s="81"/>
+      <x:c r="F16" s="81"/>
+      <x:c r="G16" s="81"/>
+      <x:c r="H16" s="81"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="74" t="str">
+        <x:v>Nguồn</x:v>
+      </x:c>
+      <x:c r="B17" s="74" t="str">
+        <x:v>Ngày</x:v>
+      </x:c>
+      <x:c r="C17" s="74" t="str">
+        <x:v>Thông tin sử dụng</x:v>
+      </x:c>
+      <x:c r="D17" s="74" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="E17" s="74" t="str">
+        <x:v>Base</x:v>
+      </x:c>
+      <x:c r="F17" s="74" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="G17" s="74" t="str">
+        <x:v>URL</x:v>
+      </x:c>
+      <x:c r="H17" s="74" t="str">
+        <x:v>Data Type</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="str">
+        <x:v>VNDIRECT Research</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>15/04/2026</x:v>
+      </x:c>
+      <x:c r="C18" t="str">
+        <x:v>Target 73k; sensitivity 66-81k; 63.250 tỷ gốc+lãi; BVPS +~10k; CAR +2-3ppt</x:v>
+      </x:c>
+      <x:c r="D18" t="n">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="E18" t="n">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="F18" t="n">
+        <x:v>81</x:v>
+      </x:c>
+      <x:c r="G18" t="str">
+        <x:v>https://www.vndirect.com.vn/STB_BCCapnhat_20260415.pdf</x:v>
+      </x:c>
+      <x:c r="H18" t="str">
+        <x:v>PUBLIC_RESEARCH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="str">
+        <x:v>HSC Research</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>19/03/2026</x:v>
+      </x:c>
+      <x:c r="C19" t="str">
+        <x:v>Target price</x:v>
+      </x:c>
+      <x:c r="D19"/>
+      <x:c r="E19" t="n">
+        <x:v>57.6</x:v>
+      </x:c>
+      <x:c r="F19"/>
+      <x:c r="G19" t="str">
+        <x:v>https://ckgvietnam.com/data/upload/bankshsc20260320en.pdf</x:v>
+      </x:c>
+      <x:c r="H19" t="str">
+        <x:v>PUBLIC_RESEARCH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
+        <x:v>MBS Research</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>15/04/2026</x:v>
+      </x:c>
+      <x:c r="C20" t="str">
+        <x:v>Target price</x:v>
+      </x:c>
+      <x:c r="D20"/>
+      <x:c r="E20" t="n">
+        <x:v>58.8</x:v>
+      </x:c>
+      <x:c r="F20"/>
+      <x:c r="G20" t="str">
+        <x:v>https://www.mbs.com.vn/files/uploads/2026/04/STB_UPDATE_20260415.pdf</x:v>
+      </x:c>
+      <x:c r="H20" t="str">
+        <x:v>PUBLIC_RESEARCH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="str">
+        <x:v>Vietcap</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>14/05/2026</x:v>
+      </x:c>
+      <x:c r="C21" t="str">
+        <x:v>Target price</x:v>
+      </x:c>
+      <x:c r="D21"/>
+      <x:c r="E21" t="n">
+        <x:v>73.5</x:v>
+      </x:c>
+      <x:c r="F21"/>
+      <x:c r="G21" t="str">
+        <x:v>https://www.vietcap.com.vn/en/research-center/stb-market-perform-0-0-positive-restructuring-progress-but-valuation-looks-full-update</x:v>
+      </x:c>
+      <x:c r="H21" t="str">
+        <x:v>PUBLIC_RESEARCH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="str">
+        <x:v>SBBS</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>14/08/2026</x:v>
+      </x:c>
+      <x:c r="C22" t="str">
+        <x:v>Target price</x:v>
+      </x:c>
+      <x:c r="D22"/>
+      <x:c r="E22" t="n">
+        <x:v>66.2</x:v>
+      </x:c>
+      <x:c r="F22"/>
+      <x:c r="G22" t="str">
+        <x:v>https://sbbs.com.vn/research-center/company-reports/2q-2026-update-stb</x:v>
+      </x:c>
+      <x:c r="H22" t="str">
+        <x:v>PUBLIC_RESEARCH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="81" t="str">
+        <x:v>Kết luận</x:v>
+      </x:c>
+      <x:c r="B24" s="81" t="str"/>
+      <x:c r="C24" s="81" t="str"/>
+      <x:c r="D24" s="81" t="str"/>
+      <x:c r="E24" s="81" t="str"/>
+      <x:c r="F24" s="81" t="str"/>
+      <x:c r="G24" s="81" t="str"/>
+      <x:c r="H24" s="81" t="str"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" t="str">
+        <x:v>80.000 đồng/cp</x:v>
+      </x:c>
+      <x:c r="B25" t="str">
+        <x:v>Hợp lý tương đối cao</x:v>
+      </x:c>
+      <x:c r="C25" t="str">
+        <x:v>Premium thị giá thấp; gần high-case standalone 81k; phù hợp nếu kỳ vọng xử lý 32,5% tích cực.</x:v>
+      </x:c>
+      <x:c r="D25" t="str"/>
+      <x:c r="E25" t="str"/>
+      <x:c r="F25" t="str"/>
+      <x:c r="G25" t="str"/>
+      <x:c r="H25" t="str"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" t="str">
+        <x:v>90.000 đồng/cp</x:v>
+      </x:c>
+      <x:c r="B26" t="str">
+        <x:v>Hợp lý có điều kiện</x:v>
+      </x:c>
+      <x:c r="C26" t="str">
+        <x:v>Cần premium chiến lược và xác suất tái cơ cấu cao hơn kịch bản standalone.</x:v>
+      </x:c>
+      <x:c r="D26" t="str"/>
+      <x:c r="E26" t="str"/>
+      <x:c r="F26" t="str"/>
+      <x:c r="G26" t="str"/>
+      <x:c r="H26" t="str"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" t="str">
+        <x:v>100.000 đồng/cp</x:v>
+      </x:c>
+      <x:c r="B27" t="str">
+        <x:v>Hợp lý có điều kiện mạnh</x:v>
+      </x:c>
+      <x:c r="C27" t="str">
+        <x:v>Giá trị lô tiến gần thu hồi đủ 63.250 tỷ; cần scarcity/quyền ảnh hưởng, hậu tái cơ cấu và/hoặc synergy để bù rủi ro thời gian.</x:v>
+      </x:c>
+      <x:c r="D27" t="str"/>
+      <x:c r="E27" t="str"/>
+      <x:c r="F27" t="str"/>
+      <x:c r="G27" t="str"/>
+      <x:c r="H27" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H1"/>
+    <x:mergeCell ref="A16:H16"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
@@ -3000,7 +3746,7 @@
     <x:mergeCell ref="A1:J1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd2cf79e99574d91"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8531a3c5b0b843f6"/>
 </x:worksheet>
 </file>
 

</xml_diff>